<commit_message>
Update internship tracker UI
</commit_message>
<xml_diff>
--- a/data/internships.xlsx
+++ b/data/internships.xlsx
@@ -460,7 +460,7 @@
         <v>Aarhus, DK</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -501,7 +501,7 @@
         <v>Trondheim, NO</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -542,7 +542,7 @@
         <v>Kongsberg, NO</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H4" t="str">
         <v/>
@@ -583,7 +583,7 @@
         <v>Solna, SE</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -624,7 +624,7 @@
         <v>Fornebu, NO</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -665,7 +665,7 @@
         <v>Lund, SE</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -706,7 +706,7 @@
         <v>Stockholm, SE</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -747,7 +747,7 @@
         <v>Södertälje, SE</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -788,7 +788,7 @@
         <v>Gothenburg, SE</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -829,7 +829,7 @@
         <v>Espoo, FI</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -870,7 +870,7 @@
         <v>Geneva, CH</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -911,7 +911,7 @@
         <v>Augsburg, DE</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -952,7 +952,7 @@
         <v>Friedrichshafen, DE</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H14" t="str">
         <v/>
@@ -993,7 +993,7 @@
         <v>Hanover, DE</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H15" t="str">
         <v/>
@@ -1034,7 +1034,7 @@
         <v>London, UK</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H16" t="str">
         <v/>
@@ -1075,7 +1075,7 @@
         <v>Bucharest, RO</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H17" t="str">
         <v/>
@@ -1116,7 +1116,7 @@
         <v>Cambridge, UK</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -1157,7 +1157,7 @@
         <v>Abingdon, UK</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -1198,7 +1198,7 @@
         <v>Bilbao, ES</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -1239,7 +1239,7 @@
         <v>Bochum, DE</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -1280,7 +1280,7 @@
         <v>Tettnang, DE</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -1321,7 +1321,7 @@
         <v>Bratislava, SK</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -1362,7 +1362,7 @@
         <v>Manchester, UK</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H24" t="str">
         <v/>
@@ -1403,7 +1403,7 @@
         <v>Helsinki, FI</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -1444,7 +1444,7 @@
         <v>Zurich, CH</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H26" t="str">
         <v/>
@@ -1485,7 +1485,7 @@
         <v>Munich, DE</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -1526,7 +1526,7 @@
         <v>Stockholm, SE</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -1567,7 +1567,7 @@
         <v>Munich, DE</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -1608,7 +1608,7 @@
         <v>Gerlingen, DE</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H30" t="str">
         <v/>
@@ -1649,7 +1649,7 @@
         <v>Neubiberg, DE</v>
       </c>
       <c r="G31">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H31" t="str">
         <v/>

</xml_diff>

<commit_message>
Refactor tracker flows and update changelog
</commit_message>
<xml_diff>
--- a/data/internships.xlsx
+++ b/data/internships.xlsx
@@ -472,13 +472,13 @@
         <v>High</v>
       </c>
       <c r="K2" t="str">
-        <v>Systems,Hardware,Embedded</v>
+        <v>Embedded,Systems,Hardware</v>
       </c>
       <c r="L2" t="str">
         <v>2026-02-04 22:59:49</v>
       </c>
       <c r="M2" t="str">
-        <v>2026-02-04 22:59:49</v>
+        <v>2026-03-26 16:06:45</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Refine tracker layout and row interaction ergonomics
</commit_message>
<xml_diff>
--- a/data/internships.xlsx
+++ b/data/internships.xlsx
@@ -448,7 +448,7 @@
         <v>Vestas</v>
       </c>
       <c r="C2" t="str">
-        <v>Researching</v>
+        <v>Applied</v>
       </c>
       <c r="D2" t="str">
         <v>2026 Summer | Nordic HQ; systems/embedded fit. Initiative application.</v>
@@ -478,7 +478,7 @@
         <v>2026-02-04 22:59:49</v>
       </c>
       <c r="M2" t="str">
-        <v>2026-03-26 16:06:45</v>
+        <v>2026-03-26 20:11:30</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Update internships spreadsheet data
</commit_message>
<xml_diff>
--- a/data/internships.xlsx
+++ b/data/internships.xlsx
@@ -609,19 +609,19 @@
         <v>213</v>
       </c>
       <c r="B6" t="str">
-        <v>TU Berlin SecT</v>
+        <v>KIT Chair of Dependable Nano Computing (CDNC)</v>
       </c>
       <c r="C6" t="str">
         <v>Researching</v>
       </c>
       <c r="D6" t="str">
-        <v>2026 Summer | Security in Telecommunications chair covering hardware security, secure embedded systems, and side-channel attacks. Initiative application.</v>
+        <v>2026 Summer | Hardware security lab known for FPGA side-channel and fault-attack research with active student thesis opportunities. Initiative application.</v>
       </c>
       <c r="E6" t="str">
-        <v>https://www.tu.berlin/en/sect</v>
+        <v>https://cdnc.itec.kit.edu/</v>
       </c>
       <c r="F6" t="str">
-        <v>Berlin, DE</v>
+        <v>Karlsruhe, DE</v>
       </c>
       <c r="G6">
         <v>5</v>
@@ -636,7 +636,7 @@
         <v>High</v>
       </c>
       <c r="K6" t="str">
-        <v>Security,Hardware,Embedded,Firmware,Systems</v>
+        <v>Hardware,Security,Embedded,Systems,Firmware</v>
       </c>
       <c r="L6" t="str">
         <v>2026-03-31</v>
@@ -650,19 +650,19 @@
         <v>214</v>
       </c>
       <c r="B7" t="str">
-        <v>KIT Chair of Dependable Nano Computing (CDNC)</v>
+        <v>TU Darmstadt ImpSec</v>
       </c>
       <c r="C7" t="str">
         <v>Researching</v>
       </c>
       <c r="D7" t="str">
-        <v>2026 Summer | Hardware security lab known for FPGA side-channel and fault-attack research with active student thesis opportunities. Initiative application.</v>
+        <v>2026 Summer | Implementation security chair focused on side-channel and fault attacks, ASICs, FPGAs, and microprocessor security. Initiative application.</v>
       </c>
       <c r="E7" t="str">
-        <v>https://cdnc.itec.kit.edu/</v>
+        <v>https://www.informatik.tu-darmstadt.de/impsec/start_impsec/index.en.jsp</v>
       </c>
       <c r="F7" t="str">
-        <v>Karlsruhe, DE</v>
+        <v>Darmstadt, DE</v>
       </c>
       <c r="G7">
         <v>5</v>
@@ -677,7 +677,7 @@
         <v>High</v>
       </c>
       <c r="K7" t="str">
-        <v>Hardware,Security,Embedded,Systems,Firmware</v>
+        <v>Hardware,Security,Embedded,Firmware,Systems</v>
       </c>
       <c r="L7" t="str">
         <v>2026-03-31</v>
@@ -691,16 +691,16 @@
         <v>215</v>
       </c>
       <c r="B8" t="str">
-        <v>TU Darmstadt ImpSec</v>
+        <v>TU Darmstadt System Security Lab</v>
       </c>
       <c r="C8" t="str">
         <v>Researching</v>
       </c>
       <c r="D8" t="str">
-        <v>2026 Summer | Implementation security chair focused on side-channel and fault attacks, ASICs, FPGAs, and microprocessor security. Initiative application.</v>
+        <v>2026 Summer | Hardware-assisted security lab covering secure processors, IoT security, and practical system hardening. Initiative application.</v>
       </c>
       <c r="E8" t="str">
-        <v>https://www.informatik.tu-darmstadt.de/impsec/start_impsec/index.en.jsp</v>
+        <v>https://www.informatik.tu-darmstadt.de/systemsecurity/system_security_lab_sys/index.en.jsp</v>
       </c>
       <c r="F8" t="str">
         <v>Darmstadt, DE</v>
@@ -718,7 +718,7 @@
         <v>High</v>
       </c>
       <c r="K8" t="str">
-        <v>Hardware,Security,Embedded,Firmware,Systems</v>
+        <v>Security,Hardware,Embedded,IoT,Systems</v>
       </c>
       <c r="L8" t="str">
         <v>2026-03-31</v>
@@ -732,22 +732,22 @@
         <v>216</v>
       </c>
       <c r="B9" t="str">
-        <v>Fraunhofer FKIE</v>
+        <v>CASA / Chair for Embedded Security</v>
       </c>
       <c r="C9" t="str">
         <v>Researching</v>
       </c>
       <c r="D9" t="str">
-        <v>2026 Summer | Applied security institute doing firmware reverse engineering, vulnerability analysis, and embedded-device forensics. Initiative application.</v>
+        <v>2026 Summer | Embedded security chair focused on secure chips, cryptographic implementations, and side-channel or fault analysis. Initiative application.</v>
       </c>
       <c r="E9" t="str">
-        <v>https://www.fkie.fraunhofer.de/en.html</v>
+        <v>https://casa.rub.de/en/</v>
       </c>
       <c r="F9" t="str">
-        <v>Bonn, DE</v>
+        <v>Bochum, DE</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -759,7 +759,7 @@
         <v>High</v>
       </c>
       <c r="K9" t="str">
-        <v>Firmware,Security,Embedded,Systems,Hardware</v>
+        <v>Hardware,Embedded,Security,Firmware,Systems</v>
       </c>
       <c r="L9" t="str">
         <v>2026-03-31</v>
@@ -773,22 +773,22 @@
         <v>217</v>
       </c>
       <c r="B10" t="str">
-        <v>Fraunhofer IIS</v>
+        <v>TU Berlin SecT</v>
       </c>
       <c r="C10" t="str">
         <v>Researching</v>
       </c>
       <c r="D10" t="str">
-        <v>2026 Summer | Secure system-on-chip research around secure RISC-V, secure boot, firmware updates, and crypto accelerators. Initiative application.</v>
+        <v>2026 Summer | Security in Telecommunications chair covering hardware security, secure embedded systems, and side-channel attacks. Initiative application.</v>
       </c>
       <c r="E10" t="str">
-        <v>https://www.iis.fraunhofer.de/en.html</v>
+        <v>https://www.tu.berlin/en/sect</v>
       </c>
       <c r="F10" t="str">
-        <v>Erlangen, DE</v>
+        <v>Berlin, DE</v>
       </c>
       <c r="G10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -800,7 +800,7 @@
         <v>High</v>
       </c>
       <c r="K10" t="str">
-        <v>Hardware,Embedded,Firmware,Security,Systems</v>
+        <v>Security,Hardware,Embedded,Firmware,Systems</v>
       </c>
       <c r="L10" t="str">
         <v>2026-03-31</v>
@@ -814,22 +814,22 @@
         <v>218</v>
       </c>
       <c r="B11" t="str">
-        <v>Fraunhofer IPMS</v>
+        <v>ETH Zurich COMSEC</v>
       </c>
       <c r="C11" t="str">
         <v>Researching</v>
       </c>
       <c r="D11" t="str">
-        <v>2026 Summer | Trusted electronics work on secure manufacturing, PUF trust anchors, encrypted firmware, and secure embedded devices. Initiative application.</v>
+        <v>2026 Summer | Computer security group doing hardware-bound attack and defense research with open thesis-style student pathways. Initiative application.</v>
       </c>
       <c r="E11" t="str">
-        <v>https://www.ipms.fraunhofer.de/en.html</v>
+        <v>https://comsec.ethz.ch/</v>
       </c>
       <c r="F11" t="str">
-        <v>Dresden, DE</v>
+        <v>Zurich, CH</v>
       </c>
       <c r="G11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -841,7 +841,7 @@
         <v>High</v>
       </c>
       <c r="K11" t="str">
-        <v>Hardware,Embedded,Firmware,Security,Systems</v>
+        <v>Security,Hardware,Systems,Embedded,Firmware</v>
       </c>
       <c r="L11" t="str">
         <v>2026-03-31</v>
@@ -937,19 +937,19 @@
         <v>221</v>
       </c>
       <c r="B14" t="str">
-        <v>RWTH Aachen ICE</v>
+        <v>Fraunhofer FKIE</v>
       </c>
       <c r="C14" t="str">
         <v>Researching</v>
       </c>
       <c r="D14" t="str">
-        <v>2026 Summer | Systems-on-silicon chair working on SoC design, virtual prototyping, and embedded cybersecurity-adjacent research. Initiative application.</v>
+        <v>2026 Summer | Applied security institute doing firmware reverse engineering, vulnerability analysis, and embedded-device forensics. Initiative application.</v>
       </c>
       <c r="E14" t="str">
-        <v>https://www.ice.rwth-aachen.de/</v>
+        <v>https://www.fkie.fraunhofer.de/en.html</v>
       </c>
       <c r="F14" t="str">
-        <v>Aachen, DE</v>
+        <v>Bonn, DE</v>
       </c>
       <c r="G14">
         <v>4</v>
@@ -964,7 +964,7 @@
         <v>High</v>
       </c>
       <c r="K14" t="str">
-        <v>Embedded,Hardware,Systems,Security,Firmware</v>
+        <v>Firmware,Security,Embedded,Systems,Hardware</v>
       </c>
       <c r="L14" t="str">
         <v>2026-03-31</v>
@@ -978,19 +978,19 @@
         <v>222</v>
       </c>
       <c r="B15" t="str">
-        <v>TU Darmstadt SEEMOO</v>
+        <v>TUM Embedded Systems and IoT</v>
       </c>
       <c r="C15" t="str">
         <v>Researching</v>
       </c>
       <c r="D15" t="str">
-        <v>2026 Summer | Secure mobile networking lab with hands-on IoT, wireless security, and resilient embedded prototype work. Initiative application.</v>
+        <v>2026 Summer | Embedded systems chair focused on secure and reliable cyber-physical, autonomous, and IoT platforms. Initiative application.</v>
       </c>
       <c r="E15" t="str">
-        <v>https://www.seemoo.tu-darmstadt.de/</v>
+        <v>https://www.ce.cit.tum.de/en/esi/staff/steinhorst/</v>
       </c>
       <c r="F15" t="str">
-        <v>Darmstadt, DE</v>
+        <v>Munich, DE</v>
       </c>
       <c r="G15">
         <v>4</v>
@@ -1005,7 +1005,7 @@
         <v>High</v>
       </c>
       <c r="K15" t="str">
-        <v>IoT,Security,Embedded,Systems,Firmware</v>
+        <v>Embedded,IoT,Systems,Security,Hardware</v>
       </c>
       <c r="L15" t="str">
         <v>2026-03-31</v>
@@ -1019,19 +1019,19 @@
         <v>223</v>
       </c>
       <c r="B16" t="str">
-        <v>TUM Embedded Systems and IoT</v>
+        <v>TU Eindhoven Security Group</v>
       </c>
       <c r="C16" t="str">
         <v>Researching</v>
       </c>
       <c r="D16" t="str">
-        <v>2026 Summer | Embedded systems chair focused on secure and reliable cyber-physical, autonomous, and IoT platforms. Initiative application.</v>
+        <v>2026 Summer | Security group researching embedded systems security, PUFs, and smart-card side-channel topics. Initiative application.</v>
       </c>
       <c r="E16" t="str">
-        <v>https://www.ce.cit.tum.de/en/esi/staff/steinhorst/</v>
+        <v>https://research.tue.nl/en/organisations/security</v>
       </c>
       <c r="F16" t="str">
-        <v>Munich, DE</v>
+        <v>Eindhoven, NL</v>
       </c>
       <c r="G16">
         <v>4</v>
@@ -1046,7 +1046,7 @@
         <v>High</v>
       </c>
       <c r="K16" t="str">
-        <v>Embedded,IoT,Systems,Security,Hardware</v>
+        <v>Security,Hardware,Embedded,Systems,Firmware</v>
       </c>
       <c r="L16" t="str">
         <v>2026-03-31</v>

</xml_diff>

<commit_message>
Add collapsible sidebar and AI analysis
</commit_message>
<xml_diff>
--- a/data/internships.xlsx
+++ b/data/internships.xlsx
@@ -442,25 +442,25 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="B2" t="str">
-        <v>Fraunhofer SIT</v>
+        <v>TU Eindhoven Security Group</v>
       </c>
       <c r="C2" t="str">
         <v>Researching</v>
       </c>
       <c r="D2" t="str">
-        <v>2026 Summer | Embedded and IoT security institute working on protocol security, trusted computing, and secure firmware updates. Initiative application.</v>
+        <v>2026 Summer | Security group researching embedded systems security, PUFs, and smart-card side-channel topics. Initiative application.</v>
       </c>
       <c r="E2" t="str">
-        <v>https://www.sit.fraunhofer.de/en/</v>
+        <v>https://research.tue.nl/en/organisations/security</v>
       </c>
       <c r="F2" t="str">
-        <v>Darmstadt, DE</v>
+        <v>Eindhoven, NL</v>
       </c>
       <c r="G2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -472,7 +472,7 @@
         <v>High</v>
       </c>
       <c r="K2" t="str">
-        <v>Embedded,Firmware,Security,IoT,Systems</v>
+        <v>Security,Hardware,Embedded,Systems,Firmware</v>
       </c>
       <c r="L2" t="str">
         <v>2026-03-31</v>
@@ -483,25 +483,25 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="B3" t="str">
-        <v>Fraunhofer EMFT</v>
+        <v>TUM Embedded Systems and IoT</v>
       </c>
       <c r="C3" t="str">
         <v>Researching</v>
       </c>
       <c r="D3" t="str">
-        <v>2026 Summer | Trusted electronics team focused on tamper protection, PUF-based key generation, and secure IoT hardware. Initiative application.</v>
+        <v>2026 Summer | Embedded systems chair focused on secure and reliable cyber-physical, autonomous, and IoT platforms. Initiative application.</v>
       </c>
       <c r="E3" t="str">
-        <v>https://www.emft.fraunhofer.de/en.html</v>
+        <v>https://www.ce.cit.tum.de/en/esi/staff/steinhorst/</v>
       </c>
       <c r="F3" t="str">
         <v>Munich, DE</v>
       </c>
       <c r="G3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -513,7 +513,7 @@
         <v>High</v>
       </c>
       <c r="K3" t="str">
-        <v>Hardware,Embedded,Security,IoT,Firmware</v>
+        <v>Embedded,IoT,Systems,Security,Hardware</v>
       </c>
       <c r="L3" t="str">
         <v>2026-03-31</v>
@@ -524,25 +524,25 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="B4" t="str">
-        <v>Fraunhofer IMS</v>
+        <v>Fraunhofer FKIE</v>
       </c>
       <c r="C4" t="str">
         <v>Researching</v>
       </c>
       <c r="D4" t="str">
-        <v>2026 Summer | Trusted electronics group researching secure key memory, PUFs, encrypted firmware storage, and secure RISC-V cores. Initiative application.</v>
+        <v>2026 Summer | Applied security institute doing firmware reverse engineering, vulnerability analysis, and embedded-device forensics. Initiative application.</v>
       </c>
       <c r="E4" t="str">
-        <v>https://www.ims.fraunhofer.de/en.html</v>
+        <v>https://www.fkie.fraunhofer.de/en.html</v>
       </c>
       <c r="F4" t="str">
-        <v>Duisburg, DE</v>
+        <v>Bonn, DE</v>
       </c>
       <c r="G4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H4" t="str">
         <v/>
@@ -554,7 +554,7 @@
         <v>High</v>
       </c>
       <c r="K4" t="str">
-        <v>Hardware,Embedded,Firmware,Security,Systems</v>
+        <v>Firmware,Security,Embedded,Systems,Hardware</v>
       </c>
       <c r="L4" t="str">
         <v>2026-03-31</v>
@@ -565,25 +565,25 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="B5" t="str">
-        <v>TUM Chair of IT Security</v>
+        <v>AIT Center for Digital Safety &amp; Security</v>
       </c>
       <c r="C5" t="str">
         <v>Researching</v>
       </c>
       <c r="D5" t="str">
-        <v>2026 Summer | University chair with a strong hardware and embedded security track plus thesis and student project intake. Initiative application.</v>
+        <v>2026 Summer | Applied research center covering secure IoT, industrial control systems, dependable systems, and wireless security. Initiative application.</v>
       </c>
       <c r="E5" t="str">
-        <v>https://www.sec.in.tum.de/i20/</v>
+        <v>https://www.ait.ac.at/en/about-the-ait/center/center-for-digital-safety-security/</v>
       </c>
       <c r="F5" t="str">
-        <v>Munich, DE</v>
+        <v>Vienna, AT</v>
       </c>
       <c r="G5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -595,7 +595,7 @@
         <v>High</v>
       </c>
       <c r="K5" t="str">
-        <v>Security,Hardware,Embedded,Firmware,Systems</v>
+        <v>Security,IoT,Systems,Embedded,Hardware</v>
       </c>
       <c r="L5" t="str">
         <v>2026-03-31</v>
@@ -606,25 +606,25 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B6" t="str">
-        <v>KIT Chair of Dependable Nano Computing (CDNC)</v>
+        <v>CARIAD Information and Automotive Security</v>
       </c>
       <c r="C6" t="str">
         <v>Researching</v>
       </c>
       <c r="D6" t="str">
-        <v>2026 Summer | Hardware security lab known for FPGA side-channel and fault-attack research with active student thesis opportunities. Initiative application.</v>
+        <v>2026 Summer | Automotive security organization covering OTA, digital keys, connected vehicles, and end-to-end platform security. Initiative application.</v>
       </c>
       <c r="E6" t="str">
-        <v>https://cdnc.itec.kit.edu/</v>
+        <v>https://cariad.technology/de/en/</v>
       </c>
       <c r="F6" t="str">
-        <v>Karlsruhe, DE</v>
+        <v>Berlin, DE</v>
       </c>
       <c r="G6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -636,7 +636,7 @@
         <v>High</v>
       </c>
       <c r="K6" t="str">
-        <v>Hardware,Security,Embedded,Systems,Firmware</v>
+        <v>Security,Embedded,Firmware,Systems,IoT</v>
       </c>
       <c r="L6" t="str">
         <v>2026-03-31</v>
@@ -647,25 +647,25 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B7" t="str">
-        <v>TU Darmstadt ImpSec</v>
+        <v>ETH Zurich COMSEC</v>
       </c>
       <c r="C7" t="str">
         <v>Researching</v>
       </c>
       <c r="D7" t="str">
-        <v>2026 Summer | Implementation security chair focused on side-channel and fault attacks, ASICs, FPGAs, and microprocessor security. Initiative application.</v>
+        <v>2026 Summer | Computer security group doing hardware-bound attack and defense research with open thesis-style student pathways. Initiative application.</v>
       </c>
       <c r="E7" t="str">
-        <v>https://www.informatik.tu-darmstadt.de/impsec/start_impsec/index.en.jsp</v>
+        <v>https://comsec.ethz.ch/</v>
       </c>
       <c r="F7" t="str">
-        <v>Darmstadt, DE</v>
+        <v>Zurich, CH</v>
       </c>
       <c r="G7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -677,7 +677,7 @@
         <v>High</v>
       </c>
       <c r="K7" t="str">
-        <v>Hardware,Security,Embedded,Firmware,Systems</v>
+        <v>Security,Hardware,Systems,Embedded,Firmware</v>
       </c>
       <c r="L7" t="str">
         <v>2026-03-31</v>
@@ -688,25 +688,25 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B8" t="str">
-        <v>TU Darmstadt System Security Lab</v>
+        <v>TU Berlin SecT</v>
       </c>
       <c r="C8" t="str">
         <v>Researching</v>
       </c>
       <c r="D8" t="str">
-        <v>2026 Summer | Hardware-assisted security lab covering secure processors, IoT security, and practical system hardening. Initiative application.</v>
+        <v>2026 Summer | Security in Telecommunications chair covering hardware security, secure embedded systems, and side-channel attacks. Initiative application.</v>
       </c>
       <c r="E8" t="str">
-        <v>https://www.informatik.tu-darmstadt.de/systemsecurity/system_security_lab_sys/index.en.jsp</v>
+        <v>https://www.tu.berlin/en/sect</v>
       </c>
       <c r="F8" t="str">
-        <v>Darmstadt, DE</v>
+        <v>Berlin, DE</v>
       </c>
       <c r="G8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -718,7 +718,7 @@
         <v>High</v>
       </c>
       <c r="K8" t="str">
-        <v>Security,Hardware,Embedded,IoT,Systems</v>
+        <v>Security,Hardware,Embedded,Firmware,Systems</v>
       </c>
       <c r="L8" t="str">
         <v>2026-03-31</v>
@@ -747,7 +747,7 @@
         <v>Bochum, DE</v>
       </c>
       <c r="G9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -770,25 +770,25 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B10" t="str">
-        <v>TU Berlin SecT</v>
+        <v>TU Darmstadt System Security Lab</v>
       </c>
       <c r="C10" t="str">
         <v>Researching</v>
       </c>
       <c r="D10" t="str">
-        <v>2026 Summer | Security in Telecommunications chair covering hardware security, secure embedded systems, and side-channel attacks. Initiative application.</v>
+        <v>2026 Summer | Hardware-assisted security lab covering secure processors, IoT security, and practical system hardening. Initiative application.</v>
       </c>
       <c r="E10" t="str">
-        <v>https://www.tu.berlin/en/sect</v>
+        <v>https://www.informatik.tu-darmstadt.de/systemsecurity/system_security_lab_sys/index.en.jsp</v>
       </c>
       <c r="F10" t="str">
-        <v>Berlin, DE</v>
+        <v>Darmstadt, DE</v>
       </c>
       <c r="G10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -800,7 +800,7 @@
         <v>High</v>
       </c>
       <c r="K10" t="str">
-        <v>Security,Hardware,Embedded,Firmware,Systems</v>
+        <v>Security,Hardware,Embedded,IoT,Systems</v>
       </c>
       <c r="L10" t="str">
         <v>2026-03-31</v>
@@ -811,25 +811,25 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B11" t="str">
-        <v>ETH Zurich COMSEC</v>
+        <v>TU Darmstadt ImpSec</v>
       </c>
       <c r="C11" t="str">
         <v>Researching</v>
       </c>
       <c r="D11" t="str">
-        <v>2026 Summer | Computer security group doing hardware-bound attack and defense research with open thesis-style student pathways. Initiative application.</v>
+        <v>2026 Summer | Implementation security chair focused on side-channel and fault attacks, ASICs, FPGAs, and microprocessor security. Initiative application.</v>
       </c>
       <c r="E11" t="str">
-        <v>https://comsec.ethz.ch/</v>
+        <v>https://www.informatik.tu-darmstadt.de/impsec/start_impsec/index.en.jsp</v>
       </c>
       <c r="F11" t="str">
-        <v>Zurich, CH</v>
+        <v>Darmstadt, DE</v>
       </c>
       <c r="G11">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -841,7 +841,7 @@
         <v>High</v>
       </c>
       <c r="K11" t="str">
-        <v>Security,Hardware,Systems,Embedded,Firmware</v>
+        <v>Hardware,Security,Embedded,Firmware,Systems</v>
       </c>
       <c r="L11" t="str">
         <v>2026-03-31</v>
@@ -852,25 +852,25 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B12" t="str">
-        <v>CARIAD Information and Automotive Security</v>
+        <v>KIT Chair of Dependable Nano Computing (CDNC)</v>
       </c>
       <c r="C12" t="str">
         <v>Researching</v>
       </c>
       <c r="D12" t="str">
-        <v>2026 Summer | Automotive security organization covering OTA, digital keys, connected vehicles, and end-to-end platform security. Initiative application.</v>
+        <v>2026 Summer | Hardware security lab known for FPGA side-channel and fault-attack research with active student thesis opportunities. Initiative application.</v>
       </c>
       <c r="E12" t="str">
-        <v>https://cariad.technology/de/en/</v>
+        <v>https://cdnc.itec.kit.edu/</v>
       </c>
       <c r="F12" t="str">
-        <v>Berlin, DE</v>
+        <v>Karlsruhe, DE</v>
       </c>
       <c r="G12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -882,7 +882,7 @@
         <v>High</v>
       </c>
       <c r="K12" t="str">
-        <v>Security,Embedded,Firmware,Systems,IoT</v>
+        <v>Hardware,Security,Embedded,Systems,Firmware</v>
       </c>
       <c r="L12" t="str">
         <v>2026-03-31</v>
@@ -893,25 +893,25 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="B13" t="str">
-        <v>AIT Center for Digital Safety &amp; Security</v>
+        <v>TUM Chair of IT Security</v>
       </c>
       <c r="C13" t="str">
         <v>Researching</v>
       </c>
       <c r="D13" t="str">
-        <v>2026 Summer | Applied research center covering secure IoT, industrial control systems, dependable systems, and wireless security. Initiative application.</v>
+        <v>2026 Summer | University chair with a strong hardware and embedded security track plus thesis and student project intake. Initiative application.</v>
       </c>
       <c r="E13" t="str">
-        <v>https://www.ait.ac.at/en/about-the-ait/center/center-for-digital-safety-security/</v>
+        <v>https://www.sec.in.tum.de/i20/</v>
       </c>
       <c r="F13" t="str">
-        <v>Vienna, AT</v>
+        <v>Munich, DE</v>
       </c>
       <c r="G13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -923,7 +923,7 @@
         <v>High</v>
       </c>
       <c r="K13" t="str">
-        <v>Security,IoT,Systems,Embedded,Hardware</v>
+        <v>Security,Hardware,Embedded,Firmware,Systems</v>
       </c>
       <c r="L13" t="str">
         <v>2026-03-31</v>
@@ -934,25 +934,25 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="B14" t="str">
-        <v>Fraunhofer FKIE</v>
+        <v>Fraunhofer IMS</v>
       </c>
       <c r="C14" t="str">
         <v>Researching</v>
       </c>
       <c r="D14" t="str">
-        <v>2026 Summer | Applied security institute doing firmware reverse engineering, vulnerability analysis, and embedded-device forensics. Initiative application.</v>
+        <v>2026 Summer | Trusted electronics group researching secure key memory, PUFs, encrypted firmware storage, and secure RISC-V cores. Initiative application.</v>
       </c>
       <c r="E14" t="str">
-        <v>https://www.fkie.fraunhofer.de/en.html</v>
+        <v>https://www.ims.fraunhofer.de/en.html</v>
       </c>
       <c r="F14" t="str">
-        <v>Bonn, DE</v>
+        <v>Duisburg, DE</v>
       </c>
       <c r="G14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H14" t="str">
         <v/>
@@ -964,7 +964,7 @@
         <v>High</v>
       </c>
       <c r="K14" t="str">
-        <v>Firmware,Security,Embedded,Systems,Hardware</v>
+        <v>Hardware,Embedded,Firmware,Security,Systems</v>
       </c>
       <c r="L14" t="str">
         <v>2026-03-31</v>
@@ -975,25 +975,25 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="B15" t="str">
-        <v>TUM Embedded Systems and IoT</v>
+        <v>Fraunhofer EMFT</v>
       </c>
       <c r="C15" t="str">
         <v>Researching</v>
       </c>
       <c r="D15" t="str">
-        <v>2026 Summer | Embedded systems chair focused on secure and reliable cyber-physical, autonomous, and IoT platforms. Initiative application.</v>
+        <v>2026 Summer | Trusted electronics team focused on tamper protection, PUF-based key generation, and secure IoT hardware. Initiative application.</v>
       </c>
       <c r="E15" t="str">
-        <v>https://www.ce.cit.tum.de/en/esi/staff/steinhorst/</v>
+        <v>https://www.emft.fraunhofer.de/en.html</v>
       </c>
       <c r="F15" t="str">
         <v>Munich, DE</v>
       </c>
       <c r="G15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H15" t="str">
         <v/>
@@ -1005,7 +1005,7 @@
         <v>High</v>
       </c>
       <c r="K15" t="str">
-        <v>Embedded,IoT,Systems,Security,Hardware</v>
+        <v>Hardware,Embedded,Security,IoT,Firmware</v>
       </c>
       <c r="L15" t="str">
         <v>2026-03-31</v>
@@ -1016,25 +1016,25 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>223</v>
+        <v>209</v>
       </c>
       <c r="B16" t="str">
-        <v>TU Eindhoven Security Group</v>
+        <v>Fraunhofer SIT</v>
       </c>
       <c r="C16" t="str">
         <v>Researching</v>
       </c>
       <c r="D16" t="str">
-        <v>2026 Summer | Security group researching embedded systems security, PUFs, and smart-card side-channel topics. Initiative application.</v>
+        <v>2026 Summer | Embedded and IoT security institute working on protocol security, trusted computing, and secure firmware updates. Initiative application.</v>
       </c>
       <c r="E16" t="str">
-        <v>https://research.tue.nl/en/organisations/security</v>
+        <v>https://www.sit.fraunhofer.de/en/</v>
       </c>
       <c r="F16" t="str">
-        <v>Eindhoven, NL</v>
+        <v>Darmstadt, DE</v>
       </c>
       <c r="G16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H16" t="str">
         <v/>
@@ -1046,7 +1046,7 @@
         <v>High</v>
       </c>
       <c r="K16" t="str">
-        <v>Security,Hardware,Embedded,Systems,Firmware</v>
+        <v>Embedded,Firmware,Security,IoT,Systems</v>
       </c>
       <c r="L16" t="str">
         <v>2026-03-31</v>

</xml_diff>